<commit_message>
datos: actualización automática 2026-09-28
</commit_message>
<xml_diff>
--- a/idecba/ejes48_comuna_tasas.xlsx
+++ b/idecba/ejes48_comuna_tasas.xlsx
@@ -1,34 +1,35 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29127"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA17E58D-E18A-4CEB-B7E7-4E4F07F95B53}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23865" windowHeight="7365" tabRatio="918"/>
   </bookViews>
   <sheets>
     <sheet name="AC_EJ_2026_04" sheetId="1" r:id="rId1"/>
-    <sheet name="1er. cuatr. de 2026 " sheetId="28" r:id="rId2"/>
-    <sheet name="3er. cuatr. de 2025" sheetId="31" r:id="rId3"/>
-    <sheet name="2do. cuatr. de 2025" sheetId="30" r:id="rId4"/>
-    <sheet name="1er. cuatr. de 2025" sheetId="29" r:id="rId5"/>
-    <sheet name="Ficha Técnica" sheetId="16" r:id="rId6"/>
+    <sheet name="2do. cuatr. de 2026 " sheetId="32" r:id="rId2"/>
+    <sheet name="1er. cuatr. de 2026 " sheetId="28" r:id="rId3"/>
+    <sheet name="3er. cuatr. de 2025" sheetId="31" r:id="rId4"/>
+    <sheet name="2do. cuatr. de 2025" sheetId="30" r:id="rId5"/>
+    <sheet name="1er. cuatr. de 2025" sheetId="29" r:id="rId6"/>
+    <sheet name="Ficha Técnica" sheetId="16" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'1er. cuatr. de 2025'!$A$3:$F$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'1er. cuatr. de 2026 '!$A$3:$F$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'2do. cuatr. de 2025'!$A$3:$F$20</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'3er. cuatr. de 2025'!$A$3:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'1er. cuatr. de 2025'!$A$3:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'1er. cuatr. de 2026 '!$A$3:$F$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'2do. cuatr. de 2025'!$A$3:$F$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2do. cuatr. de 2026 '!$A$3:$F$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'3er. cuatr. de 2025'!$A$3:$F$20</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">AC_EJ_2026_04!#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="5">'Ficha Técnica'!$A:$B</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="6">'Ficha Técnica'!$A:$B</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="189" uniqueCount="68">
   <si>
     <t>Locales Relevados</t>
   </si>
@@ -130,9 +131,6 @@
   </si>
   <si>
     <t>Presentar información sobre el estado de ocupación de los locales comerciales en los ejes comerciales de la Ciudad de Buenos Aires</t>
-  </si>
-  <si>
-    <t>Serie 5</t>
   </si>
   <si>
     <t>Presentar la evolución de la ocupación de locales comerciales en los ejes comerciales de la Ciudad de Buenos Aires</t>
@@ -184,9 +182,6 @@
     <t>Tasa de ocupación       (%)</t>
   </si>
   <si>
-    <t>Frentes de manzana</t>
-  </si>
-  <si>
     <t>Densidad comercial (relevados por frente)</t>
   </si>
   <si>
@@ -196,9 +191,6 @@
     <t>1er. cuatrimestre de 2026</t>
   </si>
   <si>
-    <t>Locales relevados, ocupados, densidad comercial, tasa de ocupación y variación respecto del relevamiento previo e interanual por comuna. 48 ejes comerciales. Ciudad de Buenos Aires. 1er. cuatrimestre de 2025/1er. cuatrimestre de 2026</t>
-  </si>
-  <si>
     <t>Locales relevados, ocupados, densidad comercial, tasa de ocupación y variación respecto del relevamiento previo e interanual por comuna. 48 ejes comerciales. Ciudad de Buenos Aires. 1er. cuatrimestre de 2026</t>
   </si>
   <si>
@@ -206,9 +198,6 @@
   </si>
   <si>
     <t>Cociente de la cantidad de locales sobre el total de frentes de manzana relevados</t>
-  </si>
-  <si>
-    <t>Presentar información sobre la cantidad de frentes de manzana relevados en los ejes comerciales de la Ciudad de Buenos Aires</t>
   </si>
   <si>
     <t>AC_EJ_2026_04</t>
@@ -260,24 +249,27 @@
     </r>
   </si>
   <si>
-    <t>Frentes de manzana por comuna</t>
-  </si>
-  <si>
-    <t>Corresponde a la consideración de los lados par e impar de las cuadras que componen los ejes comerciales, sin ajuste en función de la presencia de espacios verdes o construcciones que impidan el desarrollo comercial, desagregados por comuna. La cantidad de cuadras relevadas se calcula considerando intervalos de altura de a 100.</t>
-  </si>
-  <si>
     <t>. Dato no registrado</t>
+  </si>
+  <si>
+    <t>Locales relevados, ocupados, densidad comercial, tasa de ocupación y variación respecto del relevamiento previo e interanual por comuna. 48 ejes comerciales. Ciudad de Buenos Aires. 1er. cuatrimestre de 2025/2do. cuatrimestre de 2026</t>
+  </si>
+  <si>
+    <t>2do. cuatrimestre de 2026</t>
+  </si>
+  <si>
+    <t>Locales relevados, ocupados, densidad comercial, tasa de ocupación y variación respecto del relevamiento previo e interanual por comuna. 48 ejes comerciales. Ciudad de Buenos Aires. 2do. cuatrimestre de 2026</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="_-* #,##0.00\ [$€]_-;\-* #,##0.00\ [$€]_-;_-* &quot;-&quot;??\ [$€]_-;_-@_-"/>
   </numFmts>
-  <fonts count="36" x14ac:knownFonts="1">
+  <fonts count="35" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -462,13 +454,6 @@
       <sz val="10"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -1020,15 +1005,15 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="36"/>
@@ -1056,10 +1041,10 @@
     <xf numFmtId="0" fontId="25" fillId="0" borderId="17" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="justify" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="25" fillId="0" borderId="12" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1071,7 +1056,7 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="19" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="17" xfId="37" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="25" borderId="14" xfId="37" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1098,86 +1083,94 @@
     <xf numFmtId="0" fontId="27" fillId="0" borderId="18" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="3" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="36" applyFont="1"/>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="36" applyFill="1"/>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="37" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="25" borderId="20" xfId="37" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="21" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="21" xfId="37" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="25" borderId="16" xfId="37" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="36" applyFont="1"/>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="36" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="36" applyFont="1"/>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="49" fontId="31" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="30" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="22" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="25" borderId="24" xfId="37" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="34" fillId="0" borderId="0" xfId="32" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="33" fillId="0" borderId="0" xfId="32" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="15" xfId="37" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="32" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="25" xfId="37" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1188,55 +1181,55 @@
     </xf>
   </cellXfs>
   <cellStyles count="49">
-    <cellStyle name="20% - Énfasis1 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000000000000}"/>
-    <cellStyle name="20% - Énfasis2 2" xfId="2" xr:uid="{00000000-0005-0000-0000-000001000000}"/>
-    <cellStyle name="20% - Énfasis3 2" xfId="3" xr:uid="{00000000-0005-0000-0000-000002000000}"/>
-    <cellStyle name="20% - Énfasis4 2" xfId="4" xr:uid="{00000000-0005-0000-0000-000003000000}"/>
-    <cellStyle name="20% - Énfasis5 2" xfId="5" xr:uid="{00000000-0005-0000-0000-000004000000}"/>
-    <cellStyle name="20% - Énfasis6 2" xfId="6" xr:uid="{00000000-0005-0000-0000-000005000000}"/>
-    <cellStyle name="40% - Énfasis1 2" xfId="7" xr:uid="{00000000-0005-0000-0000-000006000000}"/>
-    <cellStyle name="40% - Énfasis2 2" xfId="8" xr:uid="{00000000-0005-0000-0000-000007000000}"/>
-    <cellStyle name="40% - Énfasis3 2" xfId="9" xr:uid="{00000000-0005-0000-0000-000008000000}"/>
-    <cellStyle name="40% - Énfasis4 2" xfId="10" xr:uid="{00000000-0005-0000-0000-000009000000}"/>
-    <cellStyle name="40% - Énfasis5 2" xfId="11" xr:uid="{00000000-0005-0000-0000-00000A000000}"/>
-    <cellStyle name="40% - Énfasis6 2" xfId="12" xr:uid="{00000000-0005-0000-0000-00000B000000}"/>
-    <cellStyle name="60% - Énfasis1 2" xfId="13" xr:uid="{00000000-0005-0000-0000-00000C000000}"/>
-    <cellStyle name="60% - Énfasis2 2" xfId="14" xr:uid="{00000000-0005-0000-0000-00000D000000}"/>
-    <cellStyle name="60% - Énfasis3 2" xfId="15" xr:uid="{00000000-0005-0000-0000-00000E000000}"/>
-    <cellStyle name="60% - Énfasis4 2" xfId="16" xr:uid="{00000000-0005-0000-0000-00000F000000}"/>
-    <cellStyle name="60% - Énfasis5 2" xfId="17" xr:uid="{00000000-0005-0000-0000-000010000000}"/>
-    <cellStyle name="60% - Énfasis6 2" xfId="18" xr:uid="{00000000-0005-0000-0000-000011000000}"/>
-    <cellStyle name="Buena 2" xfId="19" xr:uid="{00000000-0005-0000-0000-000012000000}"/>
-    <cellStyle name="Cálculo 2" xfId="20" xr:uid="{00000000-0005-0000-0000-000013000000}"/>
-    <cellStyle name="Celda de comprobación 2" xfId="21" xr:uid="{00000000-0005-0000-0000-000014000000}"/>
-    <cellStyle name="Celda vinculada 2" xfId="22" xr:uid="{00000000-0005-0000-0000-000015000000}"/>
-    <cellStyle name="Encabezado 4 2" xfId="23" xr:uid="{00000000-0005-0000-0000-000016000000}"/>
-    <cellStyle name="Énfasis1 2" xfId="24" xr:uid="{00000000-0005-0000-0000-000017000000}"/>
-    <cellStyle name="Énfasis2 2" xfId="25" xr:uid="{00000000-0005-0000-0000-000018000000}"/>
-    <cellStyle name="Énfasis3 2" xfId="26" xr:uid="{00000000-0005-0000-0000-000019000000}"/>
-    <cellStyle name="Énfasis4 2" xfId="27" xr:uid="{00000000-0005-0000-0000-00001A000000}"/>
-    <cellStyle name="Énfasis5 2" xfId="28" xr:uid="{00000000-0005-0000-0000-00001B000000}"/>
-    <cellStyle name="Énfasis6 2" xfId="29" xr:uid="{00000000-0005-0000-0000-00001C000000}"/>
-    <cellStyle name="Entrada 2" xfId="30" xr:uid="{00000000-0005-0000-0000-00001D000000}"/>
-    <cellStyle name="Euro" xfId="31" xr:uid="{00000000-0005-0000-0000-00001E000000}"/>
+    <cellStyle name="20% - Énfasis1 2" xfId="1"/>
+    <cellStyle name="20% - Énfasis2 2" xfId="2"/>
+    <cellStyle name="20% - Énfasis3 2" xfId="3"/>
+    <cellStyle name="20% - Énfasis4 2" xfId="4"/>
+    <cellStyle name="20% - Énfasis5 2" xfId="5"/>
+    <cellStyle name="20% - Énfasis6 2" xfId="6"/>
+    <cellStyle name="40% - Énfasis1 2" xfId="7"/>
+    <cellStyle name="40% - Énfasis2 2" xfId="8"/>
+    <cellStyle name="40% - Énfasis3 2" xfId="9"/>
+    <cellStyle name="40% - Énfasis4 2" xfId="10"/>
+    <cellStyle name="40% - Énfasis5 2" xfId="11"/>
+    <cellStyle name="40% - Énfasis6 2" xfId="12"/>
+    <cellStyle name="60% - Énfasis1 2" xfId="13"/>
+    <cellStyle name="60% - Énfasis2 2" xfId="14"/>
+    <cellStyle name="60% - Énfasis3 2" xfId="15"/>
+    <cellStyle name="60% - Énfasis4 2" xfId="16"/>
+    <cellStyle name="60% - Énfasis5 2" xfId="17"/>
+    <cellStyle name="60% - Énfasis6 2" xfId="18"/>
+    <cellStyle name="Buena 2" xfId="19"/>
+    <cellStyle name="Cálculo 2" xfId="20"/>
+    <cellStyle name="Celda de comprobación 2" xfId="21"/>
+    <cellStyle name="Celda vinculada 2" xfId="22"/>
+    <cellStyle name="Encabezado 4 2" xfId="23"/>
+    <cellStyle name="Énfasis1 2" xfId="24"/>
+    <cellStyle name="Énfasis2 2" xfId="25"/>
+    <cellStyle name="Énfasis3 2" xfId="26"/>
+    <cellStyle name="Énfasis4 2" xfId="27"/>
+    <cellStyle name="Énfasis5 2" xfId="28"/>
+    <cellStyle name="Énfasis6 2" xfId="29"/>
+    <cellStyle name="Entrada 2" xfId="30"/>
+    <cellStyle name="Euro" xfId="31"/>
     <cellStyle name="Hipervínculo" xfId="32" builtinId="8"/>
-    <cellStyle name="Incorrecto 2" xfId="33" xr:uid="{00000000-0005-0000-0000-000020000000}"/>
-    <cellStyle name="mio" xfId="34" xr:uid="{00000000-0005-0000-0000-000021000000}"/>
-    <cellStyle name="Neutral 2" xfId="35" xr:uid="{00000000-0005-0000-0000-000022000000}"/>
+    <cellStyle name="Incorrecto 2" xfId="33"/>
+    <cellStyle name="mio" xfId="34"/>
+    <cellStyle name="Neutral 2" xfId="35"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="36" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
-    <cellStyle name="Normal 2 2" xfId="37" xr:uid="{00000000-0005-0000-0000-000025000000}"/>
-    <cellStyle name="Normal 3" xfId="38" xr:uid="{00000000-0005-0000-0000-000026000000}"/>
-    <cellStyle name="Notas 2" xfId="39" xr:uid="{00000000-0005-0000-0000-000027000000}"/>
-    <cellStyle name="Pato" xfId="40" xr:uid="{00000000-0005-0000-0000-000028000000}"/>
-    <cellStyle name="Salida 2" xfId="41" xr:uid="{00000000-0005-0000-0000-000029000000}"/>
-    <cellStyle name="Texto de advertencia 2" xfId="42" xr:uid="{00000000-0005-0000-0000-00002A000000}"/>
-    <cellStyle name="Texto explicativo 2" xfId="43" xr:uid="{00000000-0005-0000-0000-00002B000000}"/>
-    <cellStyle name="Título 1 2" xfId="44" xr:uid="{00000000-0005-0000-0000-00002C000000}"/>
-    <cellStyle name="Título 2 2" xfId="45" xr:uid="{00000000-0005-0000-0000-00002D000000}"/>
-    <cellStyle name="Título 3 2" xfId="46" xr:uid="{00000000-0005-0000-0000-00002E000000}"/>
-    <cellStyle name="Título 4" xfId="47" xr:uid="{00000000-0005-0000-0000-00002F000000}"/>
-    <cellStyle name="Total 2" xfId="48" xr:uid="{00000000-0005-0000-0000-000030000000}"/>
+    <cellStyle name="Normal 2" xfId="36"/>
+    <cellStyle name="Normal 2 2" xfId="37"/>
+    <cellStyle name="Normal 3" xfId="38"/>
+    <cellStyle name="Notas 2" xfId="39"/>
+    <cellStyle name="Pato" xfId="40"/>
+    <cellStyle name="Salida 2" xfId="41"/>
+    <cellStyle name="Texto de advertencia 2" xfId="42"/>
+    <cellStyle name="Texto explicativo 2" xfId="43"/>
+    <cellStyle name="Título 1 2" xfId="44"/>
+    <cellStyle name="Título 2 2" xfId="45"/>
+    <cellStyle name="Título 3 2" xfId="46"/>
+    <cellStyle name="Título 4" xfId="47"/>
+    <cellStyle name="Total 2" xfId="48"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1252,9 +1245,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1292,9 +1285,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1329,7 +1322,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -1364,7 +1357,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1537,51 +1530,51 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.33203125" defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.28515625" defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="24" style="38" bestFit="1" customWidth="1"/>
-    <col min="2" max="10" width="11.33203125" style="38" customWidth="1"/>
+    <col min="2" max="10" width="11.28515625" style="38" customWidth="1"/>
     <col min="11" max="11" width="13" style="38" customWidth="1"/>
-    <col min="12" max="16384" width="11.33203125" style="38"/>
+    <col min="12" max="16384" width="11.28515625" style="38"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="55" t="s">
-        <v>50</v>
-      </c>
-      <c r="B1" s="55"/>
-      <c r="C1" s="55"/>
-      <c r="D1" s="55"/>
-      <c r="E1" s="55"/>
-      <c r="F1" s="55"/>
-      <c r="G1" s="55"/>
-      <c r="H1" s="55"/>
-      <c r="I1" s="55"/>
-      <c r="J1" s="55"/>
-      <c r="K1" s="55"/>
-    </row>
-    <row r="2" spans="1:11" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="50" t="s">
-        <v>49</v>
-      </c>
-      <c r="B2" s="54"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
-      <c r="K2" s="14"/>
-    </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="50" t="s">
-        <v>40</v>
-      </c>
-      <c r="B3" s="54"/>
+    <row r="1" spans="1:11" ht="31.9" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="59" t="s">
+        <v>65</v>
+      </c>
+      <c r="B1" s="59"/>
+      <c r="C1" s="59"/>
+      <c r="D1" s="59"/>
+      <c r="E1" s="59"/>
+      <c r="F1" s="59"/>
+      <c r="G1" s="59"/>
+      <c r="H1" s="59"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
+      <c r="K1" s="59"/>
+    </row>
+    <row r="2" spans="1:11" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A2" s="51" t="s">
+        <v>66</v>
+      </c>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+      <c r="F2" s="58"/>
+      <c r="G2" s="58"/>
+      <c r="H2" s="58"/>
+      <c r="I2" s="58"/>
+      <c r="J2" s="58"/>
+      <c r="K2" s="58"/>
+    </row>
+    <row r="3" spans="1:11" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A3" s="51" t="s">
+        <v>47</v>
+      </c>
+      <c r="B3" s="56"/>
       <c r="C3" s="14"/>
       <c r="D3" s="14"/>
       <c r="E3" s="14"/>
@@ -1592,11 +1585,11 @@
       <c r="J3" s="14"/>
       <c r="K3" s="14"/>
     </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="50" t="s">
+    <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="51" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="54"/>
+      <c r="B4" s="56"/>
       <c r="C4" s="14"/>
       <c r="D4" s="14"/>
       <c r="E4" s="14"/>
@@ -1607,11 +1600,11 @@
       <c r="J4" s="14"/>
       <c r="K4" s="14"/>
     </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="50" t="s">
+    <row r="5" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A5" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="B5" s="54"/>
+      <c r="B5" s="56"/>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
@@ -1622,27 +1615,44 @@
       <c r="J5" s="14"/>
       <c r="K5" s="14"/>
     </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="50" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A8" s="40"/>
+    <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A6" s="51" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="56"/>
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+      <c r="G6" s="14"/>
+      <c r="H6" s="14"/>
+      <c r="I6" s="14"/>
+      <c r="J6" s="14"/>
+      <c r="K6" s="14"/>
+    </row>
+    <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A7" s="51" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" s="57"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A8" s="39"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.2">
+      <c r="A9" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:K1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A6" location="'Ficha Técnica'!A1" display="Ficha Técnica" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="A5" location="'1er. cuatr. de 2025'!A1" display="1er. cuatrimestre de 2025" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="A4" location="'2do. cuatr. de 2025'!A1" display="2do. cuatrimestre de 2025" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="A3" location="'3er. cuatr. de 2025'!A1" display="3er. cuatrimestre de 2025" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="A2" location="'1er. cuatr. de 2026 '!A1" display="1er. cuatrimestre de 2026" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="A7" location="'Ficha Técnica'!A1" display="Ficha Técnica"/>
+    <hyperlink ref="A6" location="'1er. cuatr. de 2025'!A1" display="1er. cuatrimestre de 2025"/>
+    <hyperlink ref="A5" location="'2do. cuatr. de 2025'!A1" display="2do. cuatrimestre de 2025"/>
+    <hyperlink ref="A4" location="'3er. cuatr. de 2025'!A1" display="3er. cuatrimestre de 2025"/>
+    <hyperlink ref="A3" location="'1er. cuatr. de 2026 '!A1" display="1er. cuatrimestre de 2026"/>
+    <hyperlink ref="A2" location="'2do. cuatr. de 2026 '!A1" display="2do. cuatrimestre de 2026"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
@@ -1650,101 +1660,101 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:G19"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" customWidth="1"/>
-    <col min="2" max="4" width="11.33203125" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" customWidth="1"/>
-    <col min="8" max="9" width="11.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="8" max="9" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.85546875" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
-        <v>51</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-    </row>
-    <row r="2" spans="1:7" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="48" t="s">
+    <row r="1" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="60" t="s">
+        <v>67</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+    </row>
+    <row r="2" spans="1:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="F2" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" s="48" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="42">
-        <v>12896</v>
+        <v>12916</v>
       </c>
       <c r="C3" s="42">
-        <v>11605</v>
+        <v>11528</v>
       </c>
       <c r="D3" s="43">
-        <v>89.989143920595538</v>
+        <v>89.253638897491484</v>
       </c>
       <c r="E3" s="43">
-        <v>-1.3505986751557515</v>
+        <v>-0.73550502310405363</v>
       </c>
       <c r="F3" s="43">
-        <v>-1.5615672729727947</v>
+        <v>-2.23177018989918</v>
       </c>
       <c r="G3" s="44">
-        <v>13.807280513918629</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13.828693790149893</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="45">
         <v>1</v>
       </c>
       <c r="B4" s="1">
-        <v>1908</v>
+        <v>1910</v>
       </c>
       <c r="C4" s="2">
-        <v>1657</v>
+        <v>1658</v>
       </c>
       <c r="D4" s="3">
-        <v>86.84486373165619</v>
+        <v>86.806282722513089</v>
       </c>
       <c r="E4" s="3">
-        <v>-1.0148955566745315</v>
+        <v>-3.8581009143101141E-2</v>
       </c>
       <c r="F4" s="13">
-        <v>-0.54965103627630185</v>
+        <v>-2.0126149152821853</v>
       </c>
       <c r="G4" s="3">
-        <v>11.223529411764705</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11.235294117647058</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="45">
         <v>2</v>
       </c>
@@ -1752,45 +1762,45 @@
         <v>746</v>
       </c>
       <c r="C5" s="2">
-        <v>672</v>
+        <v>668</v>
       </c>
       <c r="D5" s="3">
-        <v>90.080428954423596</v>
+        <v>89.544235924932977</v>
       </c>
       <c r="E5" s="3">
-        <v>-1.9894635186946772</v>
+        <v>-0.53619302949061876</v>
       </c>
       <c r="F5" s="13">
-        <v>-4.5862377122430757</v>
+        <v>-3.6284548381192394</v>
       </c>
       <c r="G5" s="3">
         <v>12.03225806451613</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="45">
         <v>3</v>
       </c>
       <c r="B6" s="1">
-        <v>1251</v>
+        <v>1252</v>
       </c>
       <c r="C6" s="2">
-        <v>1161</v>
+        <v>1152</v>
       </c>
       <c r="D6" s="3">
-        <v>92.805755395683448</v>
+        <v>92.012779552715656</v>
       </c>
       <c r="E6" s="3">
-        <v>-1.3354966107370956</v>
+        <v>-0.79297584296779178</v>
       </c>
       <c r="F6" s="13">
-        <v>-1.1093767100011007</v>
+        <v>-2.0015859700297511</v>
       </c>
       <c r="G6" s="3">
-        <v>14.546511627906977</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14.55813953488372</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="45">
         <v>4</v>
       </c>
@@ -1798,91 +1808,91 @@
         <v>706</v>
       </c>
       <c r="C7" s="2">
-        <v>625</v>
+        <v>621</v>
       </c>
       <c r="D7" s="3">
-        <v>88.526912181303118</v>
+        <v>87.960339943342774</v>
       </c>
       <c r="E7" s="3">
-        <v>-0.56399690960597582</v>
+        <v>-0.56657223796034373</v>
       </c>
       <c r="F7" s="13">
-        <v>-0.25425125359993217</v>
+        <v>-1.176150307353609</v>
       </c>
       <c r="G7" s="3">
         <v>13.074074074074074</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="45">
         <v>5</v>
       </c>
       <c r="B8" s="1">
-        <v>770</v>
+        <v>773</v>
       </c>
       <c r="C8" s="2">
-        <v>707</v>
+        <v>703</v>
       </c>
       <c r="D8" s="3">
-        <v>91.818181818181827</v>
+        <v>90.944372574385511</v>
       </c>
       <c r="E8" s="3">
-        <v>-2.101611196048438</v>
+        <v>-0.87380924379631608</v>
       </c>
       <c r="F8" s="13">
-        <v>-1.9561372479660264</v>
+        <v>-2.0698576972833109</v>
       </c>
       <c r="G8" s="3">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14.054545454545455</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="45">
         <v>6</v>
       </c>
       <c r="B9" s="1">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C9" s="2">
-        <v>354</v>
+        <v>349</v>
       </c>
       <c r="D9" s="3">
-        <v>96.195652173913047</v>
+        <v>95.355191256830594</v>
       </c>
       <c r="E9" s="3">
-        <v>-0.26211349366188585</v>
+        <v>-0.84046091708245285</v>
       </c>
       <c r="F9" s="13">
-        <v>2.0788785934911402E-2</v>
+        <v>-0.81967213114754145</v>
       </c>
       <c r="G9" s="3">
-        <v>12.689655172413794</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12.620689655172415</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="45">
         <v>7</v>
       </c>
       <c r="B10" s="1">
-        <v>1201</v>
+        <v>1205</v>
       </c>
       <c r="C10" s="2">
-        <v>1109</v>
+        <v>1106</v>
       </c>
       <c r="D10" s="3">
-        <v>92.339716902581188</v>
+        <v>91.784232365145229</v>
       </c>
       <c r="E10" s="3">
-        <v>-2.0077477690730205</v>
+        <v>-0.55548453743595871</v>
       </c>
       <c r="F10" s="13">
-        <v>-0.35322234208220493</v>
+        <v>-1.6488515916295086</v>
       </c>
       <c r="G10" s="3">
-        <v>19.370967741935484</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>19.43548387096774</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="45">
         <v>8</v>
       </c>
@@ -1890,160 +1900,163 @@
         <v>507</v>
       </c>
       <c r="C11" s="2">
-        <v>442</v>
+        <v>430</v>
       </c>
       <c r="D11" s="3">
-        <v>87.179487179487182</v>
+        <v>84.812623274161737</v>
       </c>
       <c r="E11" s="3">
-        <v>-1.2063395921663584</v>
+        <v>-2.3668639053254452</v>
       </c>
       <c r="F11" s="13">
-        <v>-1.6659139946811052</v>
+        <v>-2.2967517258382628</v>
       </c>
       <c r="G11" s="3">
         <v>14.083333333333334</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="45">
         <v>9</v>
       </c>
       <c r="B12" s="1">
-        <v>535</v>
+        <v>537</v>
       </c>
       <c r="C12" s="2">
-        <v>481</v>
+        <v>476</v>
       </c>
       <c r="D12" s="3">
-        <v>89.90654205607477</v>
+        <v>88.640595903165732</v>
       </c>
       <c r="E12" s="3">
-        <v>0.56074766355139616</v>
+        <v>-1.2659461529090379</v>
       </c>
       <c r="F12" s="13">
-        <v>0.7274375784628262</v>
+        <v>-0.5385085744462117</v>
       </c>
       <c r="G12" s="3">
-        <v>15.285714285714286</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>15.342857142857143</v>
+      </c>
+      <c r="I12" s="48"/>
+    </row>
+    <row r="13" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="45">
         <v>10</v>
       </c>
       <c r="B13" s="1">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="C13" s="2">
-        <v>1058</v>
+        <v>1072</v>
       </c>
       <c r="D13" s="3">
-        <v>90.815450643776828</v>
+        <v>91.938250428816474</v>
       </c>
       <c r="E13" s="3">
-        <v>-1.8632745930879366</v>
+        <v>1.1227997850396463</v>
       </c>
       <c r="F13" s="13">
-        <v>-2.4719848123333321</v>
+        <v>-0.90657715739042999</v>
       </c>
       <c r="G13" s="3">
-        <v>17.651515151515152</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17.666666666666668</v>
+      </c>
+      <c r="I13" s="48"/>
+    </row>
+    <row r="14" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="45">
         <v>11</v>
       </c>
       <c r="B14" s="1">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="C14" s="2">
-        <v>453</v>
+        <v>454</v>
       </c>
       <c r="D14" s="3">
-        <v>93.01848049281314</v>
+        <v>92.842535787321069</v>
       </c>
       <c r="E14" s="3">
-        <v>1.0431718508378367</v>
+        <v>-0.17594470549207131</v>
       </c>
       <c r="F14" s="13">
-        <v>0.77358253362946527</v>
+        <v>-0.17594470549207131</v>
       </c>
       <c r="G14" s="3">
-        <v>15.709677419354838</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>15.774193548387096</v>
+      </c>
+      <c r="I14" s="48"/>
+    </row>
+    <row r="15" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="45">
         <v>12</v>
       </c>
       <c r="B15" s="1">
-        <v>396</v>
+        <v>397</v>
       </c>
       <c r="C15" s="2">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="D15" s="3">
-        <v>92.171717171717177</v>
+        <v>90.931989924433253</v>
       </c>
       <c r="E15" s="3">
-        <v>-1.9718596544791467E-2</v>
+        <v>-1.2397272472839234</v>
       </c>
       <c r="F15" s="13">
-        <v>-1.0443632302928734</v>
+        <v>-2.5188916876574154</v>
       </c>
       <c r="G15" s="3">
-        <v>15.84</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>15.88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="45">
         <v>13</v>
       </c>
       <c r="B16" s="1">
-        <v>844</v>
+        <v>846</v>
       </c>
       <c r="C16" s="2">
-        <v>772</v>
+        <v>752</v>
       </c>
       <c r="D16" s="3">
-        <v>91.469194312796205</v>
+        <v>88.888888888888886</v>
       </c>
       <c r="E16" s="3">
-        <v>-1.3289166671329582</v>
+        <v>-2.5803054239073191</v>
       </c>
       <c r="F16" s="13">
-        <v>-3.3237050954878242</v>
+        <v>-4.9645390070921991</v>
       </c>
       <c r="G16" s="3">
-        <v>14.305084745762711</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14.338983050847459</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="45">
         <v>14</v>
       </c>
       <c r="B17" s="1">
-        <v>718</v>
+        <v>722</v>
       </c>
       <c r="C17" s="2">
-        <v>630</v>
+        <v>626</v>
       </c>
       <c r="D17" s="3">
-        <v>87.743732590529248</v>
+        <v>86.70360110803324</v>
       </c>
       <c r="E17" s="3">
-        <v>-1.3471765003798453</v>
+        <v>-1.0401314824960082</v>
       </c>
       <c r="F17" s="13">
-        <v>-2.117378520581866</v>
+        <v>-2.989992206729994</v>
       </c>
       <c r="G17" s="3">
-        <v>11.770491803278688</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11.836065573770492</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="46">
         <v>15</v>
       </c>
@@ -2051,31 +2064,31 @@
         <v>1294</v>
       </c>
       <c r="C18" s="29">
-        <v>1119</v>
+        <v>1100</v>
       </c>
       <c r="D18" s="27">
-        <v>86.476043276661514</v>
+        <v>85.00772797527047</v>
       </c>
       <c r="E18" s="27">
-        <v>-2.9038016845787951</v>
+        <v>-1.4683153013910442</v>
       </c>
       <c r="F18" s="30">
-        <v>-3.4625127909268087</v>
+        <v>-3.9753228721871494</v>
       </c>
       <c r="G18" s="27">
         <v>12.563106796116505</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="57" t="s">
-        <v>36</v>
-      </c>
-      <c r="B19" s="57"/>
-      <c r="C19" s="57"/>
-      <c r="D19" s="57"/>
-      <c r="E19" s="57"/>
-      <c r="F19" s="57"/>
-      <c r="G19" s="57"/>
+    <row r="19" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="61"/>
+      <c r="C19" s="61"/>
+      <c r="D19" s="61"/>
+      <c r="E19" s="61"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2088,262 +2101,262 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I19"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" customWidth="1"/>
-    <col min="2" max="4" width="11.33203125" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" customWidth="1"/>
-    <col min="8" max="9" width="11.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="8" max="9" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.85546875" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
-        <v>57</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-    </row>
-    <row r="2" spans="1:7" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
+    <row r="1" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="B2" s="48" t="s">
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+    </row>
+    <row r="2" spans="1:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="F2" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" s="48" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="42">
-        <v>12898</v>
+        <v>12896</v>
       </c>
       <c r="C3" s="42">
-        <v>11781</v>
+        <v>11605</v>
       </c>
       <c r="D3" s="43">
-        <v>91.339742595751289</v>
+        <v>89.989143920595538</v>
       </c>
       <c r="E3" s="43">
-        <v>-0.14566649163937484</v>
-      </c>
-      <c r="F3" s="44" t="s">
-        <v>60</v>
+        <v>-1.3505986751557515</v>
+      </c>
+      <c r="F3" s="43">
+        <v>-1.5615672729727947</v>
       </c>
       <c r="G3" s="44">
-        <v>13.809421841541756</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13.807280513918629</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="45">
         <v>1</v>
       </c>
       <c r="B4" s="1">
-        <v>1911</v>
+        <v>1908</v>
       </c>
       <c r="C4" s="2">
-        <v>1679</v>
+        <v>1657</v>
       </c>
       <c r="D4" s="3">
-        <v>87.859759288330721</v>
+        <v>86.84486373165619</v>
       </c>
       <c r="E4" s="3">
-        <v>-0.95913834946455268</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>60</v>
+        <v>-1.0148955566745315</v>
+      </c>
+      <c r="F4" s="13">
+        <v>-0.54965103627630185</v>
       </c>
       <c r="G4" s="3">
-        <v>11.241176470588234</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11.223529411764705</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="45">
         <v>2</v>
       </c>
       <c r="B5" s="1">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="C5" s="2">
-        <v>685</v>
+        <v>672</v>
       </c>
       <c r="D5" s="3">
-        <v>92.069892473118273</v>
+        <v>90.080428954423596</v>
       </c>
       <c r="E5" s="3">
-        <v>-1.1027982899339435</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>60</v>
+        <v>-1.9894635186946772</v>
+      </c>
+      <c r="F5" s="13">
+        <v>-4.5862377122430757</v>
       </c>
       <c r="G5" s="3">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12.03225806451613</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="45">
         <v>3</v>
       </c>
       <c r="B6" s="1">
-        <v>1246</v>
+        <v>1251</v>
       </c>
       <c r="C6" s="2">
-        <v>1173</v>
+        <v>1161</v>
       </c>
       <c r="D6" s="3">
-        <v>94.141252006420544</v>
+        <v>92.805755395683448</v>
       </c>
       <c r="E6" s="3">
-        <v>0.12688648367513622</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>60</v>
+        <v>-1.3354966107370956</v>
+      </c>
+      <c r="F6" s="13">
+        <v>-1.1093767100011007</v>
       </c>
       <c r="G6" s="3">
-        <v>14.488372093023257</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14.546511627906977</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="45">
         <v>4</v>
       </c>
       <c r="B7" s="1">
-        <v>715</v>
+        <v>706</v>
       </c>
       <c r="C7" s="2">
-        <v>637</v>
+        <v>625</v>
       </c>
       <c r="D7" s="3">
-        <v>89.090909090909093</v>
+        <v>88.526912181303118</v>
       </c>
       <c r="E7" s="3">
-        <v>-4.5581159787289494E-2</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>60</v>
+        <v>-0.56399690960597582</v>
+      </c>
+      <c r="F7" s="13">
+        <v>-0.25425125359993217</v>
       </c>
       <c r="G7" s="3">
-        <v>13.24074074074074</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>13.074074074074074</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="45">
         <v>5</v>
       </c>
       <c r="B8" s="1">
-        <v>773</v>
+        <v>770</v>
       </c>
       <c r="C8" s="2">
-        <v>726</v>
+        <v>707</v>
       </c>
       <c r="D8" s="3">
-        <v>93.919793014230265</v>
+        <v>91.818181818181827</v>
       </c>
       <c r="E8" s="3">
-        <v>0.9055627425614432</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>60</v>
+        <v>-2.101611196048438</v>
+      </c>
+      <c r="F8" s="13">
+        <v>-1.9561372479660264</v>
       </c>
       <c r="G8" s="3">
-        <v>14.054545454545455</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="45">
         <v>6</v>
       </c>
       <c r="B9" s="1">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="C9" s="2">
         <v>354</v>
       </c>
       <c r="D9" s="3">
-        <v>96.457765667574932</v>
+        <v>96.195652173913047</v>
       </c>
       <c r="E9" s="3">
-        <v>0.28290227959679726</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>60</v>
+        <v>-0.26211349366188585</v>
+      </c>
+      <c r="F9" s="13">
+        <v>2.0788785934911402E-2</v>
       </c>
       <c r="G9" s="3">
-        <v>12.655172413793103</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>12.689655172413794</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="45">
         <v>7</v>
       </c>
       <c r="B10" s="1">
-        <v>1203</v>
+        <v>1201</v>
       </c>
       <c r="C10" s="2">
-        <v>1135</v>
+        <v>1109</v>
       </c>
       <c r="D10" s="3">
-        <v>94.347464671654208</v>
+        <v>92.339716902581188</v>
       </c>
       <c r="E10" s="3">
-        <v>0.9143807148794707</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>60</v>
+        <v>-2.0077477690730205</v>
+      </c>
+      <c r="F10" s="13">
+        <v>-0.35322234208220493</v>
       </c>
       <c r="G10" s="3">
-        <v>19.403225806451612</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>19.370967741935484</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="45">
         <v>8</v>
       </c>
       <c r="B11" s="1">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C11" s="2">
-        <v>449</v>
+        <v>442</v>
       </c>
       <c r="D11" s="3">
-        <v>88.385826771653541</v>
+        <v>87.179487179487182</v>
       </c>
       <c r="E11" s="3">
-        <v>1.2764517716535408</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>60</v>
+        <v>-1.2063395921663584</v>
+      </c>
+      <c r="F11" s="13">
+        <v>-1.6659139946811052</v>
       </c>
       <c r="G11" s="3">
-        <v>14.111111111111111</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14.083333333333334</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="45">
         <v>9</v>
       </c>
@@ -2351,185 +2364,176 @@
         <v>535</v>
       </c>
       <c r="C12" s="2">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="D12" s="3">
-        <v>89.345794392523374</v>
+        <v>89.90654205607477</v>
       </c>
       <c r="E12" s="3">
-        <v>0.16668991491143004</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>60</v>
+        <v>0.56074766355139616</v>
+      </c>
+      <c r="F12" s="13">
+        <v>0.7274375784628262</v>
       </c>
       <c r="G12" s="3">
         <v>15.285714285714286</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I12" s="48"/>
+    </row>
+    <row r="13" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="45">
         <v>10</v>
       </c>
       <c r="B13" s="1">
-        <v>1161</v>
+        <v>1165</v>
       </c>
       <c r="C13" s="2">
-        <v>1076</v>
+        <v>1058</v>
       </c>
       <c r="D13" s="3">
-        <v>92.678725236864764</v>
+        <v>90.815450643776828</v>
       </c>
       <c r="E13" s="3">
-        <v>-0.16610234934213963</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>60</v>
+        <v>-1.8632745930879366</v>
+      </c>
+      <c r="F13" s="13">
+        <v>-2.4719848123333321</v>
       </c>
       <c r="G13" s="3">
-        <v>17.59090909090909</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>17.651515151515152</v>
+      </c>
+      <c r="I13" s="48"/>
+    </row>
+    <row r="14" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="45">
         <v>11</v>
       </c>
       <c r="B14" s="1">
-        <v>486</v>
+        <v>487</v>
       </c>
       <c r="C14" s="2">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="D14" s="3">
-        <v>91.975308641975303</v>
+        <v>93.01848049281314</v>
       </c>
       <c r="E14" s="3">
-        <v>-1.0431718508378367</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>60</v>
+        <v>1.0431718508378367</v>
+      </c>
+      <c r="F14" s="13">
+        <v>0.77358253362946527</v>
       </c>
       <c r="G14" s="3">
-        <v>15.67741935483871</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>15.709677419354838</v>
+      </c>
+      <c r="I14" s="48"/>
+    </row>
+    <row r="15" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="45">
         <v>12</v>
       </c>
       <c r="B15" s="1">
-        <v>397</v>
+        <v>396</v>
       </c>
       <c r="C15" s="2">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="D15" s="3">
-        <v>92.191435768261968</v>
+        <v>92.171717171717177</v>
       </c>
       <c r="E15" s="3">
-        <v>-1.2594458438287006</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>60</v>
+        <v>-1.9718596544791467E-2</v>
+      </c>
+      <c r="F15" s="13">
+        <v>-1.0443632302928734</v>
       </c>
       <c r="G15" s="3">
-        <v>15.88</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>15.84</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="45">
         <v>13</v>
       </c>
       <c r="B16" s="1">
-        <v>847</v>
+        <v>844</v>
       </c>
       <c r="C16" s="2">
-        <v>786</v>
+        <v>772</v>
       </c>
       <c r="D16" s="3">
-        <v>92.798110979929163</v>
+        <v>91.469194312796205</v>
       </c>
       <c r="E16" s="3">
-        <v>-1.0553169160519218</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>60</v>
+        <v>-1.3289166671329582</v>
+      </c>
+      <c r="F16" s="13">
+        <v>-3.3237050954878242</v>
       </c>
       <c r="G16" s="3">
-        <v>14.35593220338983</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>14.305084745762711</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="45">
         <v>14</v>
       </c>
       <c r="B17" s="1">
-        <v>715</v>
+        <v>718</v>
       </c>
       <c r="C17" s="2">
-        <v>637</v>
+        <v>630</v>
       </c>
       <c r="D17" s="3">
-        <v>89.090909090909093</v>
+        <v>87.743732590529248</v>
       </c>
       <c r="E17" s="3">
-        <v>-0.60268422385414055</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>60</v>
+        <v>-1.3471765003798453</v>
+      </c>
+      <c r="F17" s="13">
+        <v>-2.117378520581866</v>
       </c>
       <c r="G17" s="3">
-        <v>11.721311475409836</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+        <v>11.770491803278688</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="46">
         <v>15</v>
       </c>
       <c r="B18" s="28">
-        <v>1290</v>
+        <v>1294</v>
       </c>
       <c r="C18" s="29">
-        <v>1153</v>
+        <v>1119</v>
       </c>
       <c r="D18" s="27">
-        <v>89.379844961240309</v>
+        <v>86.476043276661514</v>
       </c>
       <c r="E18" s="27">
-        <v>0.39679411378268981</v>
-      </c>
-      <c r="F18" s="27" t="s">
-        <v>60</v>
+        <v>-2.9038016845787951</v>
+      </c>
+      <c r="F18" s="30">
+        <v>-3.4625127909268087</v>
       </c>
       <c r="G18" s="27">
-        <v>12.524271844660195</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="58" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19" s="58"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="58"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="58"/>
-    </row>
-    <row r="20" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="57" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="57"/>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
+        <v>12.563106796116505</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="61"/>
+      <c r="C19" s="61"/>
+      <c r="D19" s="61"/>
+      <c r="E19" s="61"/>
+      <c r="F19" s="61"/>
+      <c r="G19" s="61"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="2">
     <mergeCell ref="A1:G1"/>
-    <mergeCell ref="A20:G20"/>
     <mergeCell ref="A19:G19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2538,444 +2542,446 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:K20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" customWidth="1"/>
-    <col min="2" max="4" width="11.33203125" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" customWidth="1"/>
-    <col min="8" max="9" width="11.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="8" max="9" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.85546875" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
-        <v>58</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-    </row>
-    <row r="2" spans="1:7" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="48" t="s">
+    <row r="1" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="60" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+    </row>
+    <row r="2" spans="1:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="F2" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" s="48" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="42">
-        <v>12919</v>
+        <v>12898</v>
       </c>
       <c r="C3" s="42">
-        <v>11819</v>
+        <v>11781</v>
       </c>
       <c r="D3" s="43">
-        <v>91.485409087390664</v>
+        <v>91.339742595751289</v>
       </c>
       <c r="E3" s="43">
-        <v>-6.5302106177668406E-2</v>
+        <v>-0.14566649163937484</v>
       </c>
       <c r="F3" s="44" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G3" s="44">
-        <v>13.831905781584583</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="52">
+        <v>13.809421841541756</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="45">
         <v>1</v>
       </c>
       <c r="B4" s="1">
-        <v>1905</v>
+        <v>1911</v>
       </c>
       <c r="C4" s="2">
-        <v>1692</v>
+        <v>1679</v>
       </c>
       <c r="D4" s="3">
-        <v>88.818897637795274</v>
+        <v>87.859759288330721</v>
       </c>
       <c r="E4" s="3">
-        <v>1.4243828698627823</v>
+        <v>-0.95913834946455268</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G4" s="3">
-        <v>11.205882352941176</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="52">
+        <v>11.241176470588234</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="45">
         <v>2</v>
       </c>
       <c r="B5" s="1">
-        <v>747</v>
+        <v>744</v>
       </c>
       <c r="C5" s="2">
-        <v>696</v>
+        <v>685</v>
       </c>
       <c r="D5" s="3">
-        <v>93.172690763052216</v>
+        <v>92.069892473118273</v>
       </c>
       <c r="E5" s="3">
-        <v>-1.4939759036144551</v>
+        <v>-1.1027982899339435</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G5" s="3">
-        <v>12.048387096774194</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="52">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="45">
         <v>3</v>
       </c>
       <c r="B6" s="1">
-        <v>1253</v>
+        <v>1246</v>
       </c>
       <c r="C6" s="2">
-        <v>1178</v>
+        <v>1173</v>
       </c>
       <c r="D6" s="3">
-        <v>94.014365522745408</v>
+        <v>94.141252006420544</v>
       </c>
       <c r="E6" s="3">
-        <v>9.9233417060858642E-2</v>
+        <v>0.12688648367513622</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G6" s="3">
-        <v>14.569767441860465</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="52">
+        <v>14.488372093023257</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="45">
         <v>4</v>
       </c>
       <c r="B7" s="1">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="C7" s="2">
-        <v>640</v>
+        <v>637</v>
       </c>
       <c r="D7" s="3">
-        <v>89.136490250696383</v>
+        <v>89.090909090909093</v>
       </c>
       <c r="E7" s="3">
-        <v>0.35532681579333314</v>
+        <v>-4.5581159787289494E-2</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G7" s="3">
-        <v>13.296296296296296</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="52">
+        <v>13.24074074074074</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="45">
         <v>5</v>
       </c>
       <c r="B8" s="1">
         <v>773</v>
       </c>
       <c r="C8" s="2">
-        <v>719</v>
+        <v>726</v>
       </c>
       <c r="D8" s="3">
-        <v>93.014230271668822</v>
+        <v>93.919793014230265</v>
       </c>
       <c r="E8" s="3">
-        <v>-0.76008879447903155</v>
+        <v>0.9055627425614432</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G8" s="3">
         <v>14.054545454545455</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="52">
+    <row r="9" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="45">
         <v>6</v>
       </c>
       <c r="B9" s="1">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="C9" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="D9" s="3">
-        <v>96.174863387978135</v>
+        <v>96.457765667574932</v>
       </c>
       <c r="E9" s="3">
-        <v>0</v>
+        <v>0.28290227959679726</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G9" s="3">
-        <v>12.620689655172415</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="52">
+        <v>12.655172413793103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="45">
         <v>7</v>
       </c>
       <c r="B10" s="1">
         <v>1203</v>
       </c>
       <c r="C10" s="2">
-        <v>1124</v>
+        <v>1135</v>
       </c>
       <c r="D10" s="3">
-        <v>93.433083956774738</v>
+        <v>94.347464671654208</v>
       </c>
       <c r="E10" s="3">
-        <v>0.74014471211134492</v>
+        <v>0.9143807148794707</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G10" s="3">
         <v>19.403225806451612</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="52">
+    <row r="11" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="45">
         <v>8</v>
       </c>
       <c r="B11" s="1">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="C11" s="2">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="D11" s="3">
-        <v>87.109375</v>
+        <v>88.385826771653541</v>
       </c>
       <c r="E11" s="3">
-        <v>-1.7360261741682876</v>
+        <v>1.2764517716535408</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G11" s="3">
-        <v>14.222222222222221</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="52">
+        <v>14.111111111111111</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="45">
         <v>9</v>
       </c>
       <c r="B12" s="1">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="C12" s="2">
         <v>478</v>
       </c>
       <c r="D12" s="3">
-        <v>89.179104477611943</v>
+        <v>89.345794392523374</v>
       </c>
       <c r="E12" s="3">
-        <v>0</v>
+        <v>0.16668991491143004</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G12" s="3">
-        <v>15.314285714285715</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="52">
+        <v>15.285714285714286</v>
+      </c>
+      <c r="I12" s="48"/>
+    </row>
+    <row r="13" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="45">
         <v>10</v>
       </c>
       <c r="B13" s="1">
-        <v>1160</v>
+        <v>1161</v>
       </c>
       <c r="C13" s="2">
-        <v>1077</v>
+        <v>1076</v>
       </c>
       <c r="D13" s="3">
-        <v>92.844827586206904</v>
+        <v>92.678725236864764</v>
       </c>
       <c r="E13" s="3">
-        <v>-0.44260786990325585</v>
+        <v>-0.16610234934213963</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G13" s="3">
-        <v>17.575757575757574</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="52">
+        <v>17.59090909090909</v>
+      </c>
+      <c r="I13" s="48"/>
+    </row>
+    <row r="14" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="45">
         <v>11</v>
       </c>
       <c r="B14" s="1">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="C14" s="2">
-        <v>453</v>
+        <v>447</v>
       </c>
       <c r="D14" s="3">
-        <v>93.01848049281314</v>
+        <v>91.975308641975303</v>
       </c>
       <c r="E14" s="3">
-        <v>0.77358253362946527</v>
+        <v>-1.0431718508378367</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G14" s="3">
-        <v>15.709677419354838</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="52">
+        <v>15.67741935483871</v>
+      </c>
+      <c r="I14" s="48"/>
+    </row>
+    <row r="15" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="45">
         <v>12</v>
       </c>
       <c r="B15" s="1">
         <v>397</v>
       </c>
       <c r="C15" s="2">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="D15" s="3">
-        <v>93.450881612090669</v>
+        <v>92.191435768261968</v>
       </c>
       <c r="E15" s="3">
-        <v>0.23480121008061872</v>
+        <v>-1.2594458438287006</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G15" s="3">
         <v>15.88</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="52">
+    <row r="16" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="45">
         <v>13</v>
       </c>
       <c r="B16" s="1">
-        <v>846</v>
+        <v>847</v>
       </c>
       <c r="C16" s="2">
-        <v>794</v>
+        <v>786</v>
       </c>
       <c r="D16" s="3">
-        <v>93.853427895981085</v>
+        <v>92.798110979929163</v>
       </c>
       <c r="E16" s="3">
-        <v>-0.93947151230294423</v>
+        <v>-1.0553169160519218</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G16" s="3">
-        <v>14.338983050847459</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="52">
+        <v>14.35593220338983</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="45">
         <v>14</v>
       </c>
       <c r="B17" s="1">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="C17" s="2">
-        <v>644</v>
+        <v>637</v>
       </c>
       <c r="D17" s="3">
-        <v>89.693593314763234</v>
+        <v>89.090909090909093</v>
       </c>
       <c r="E17" s="3">
-        <v>-0.16751779634788022</v>
+        <v>-0.60268422385414055</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G17" s="3">
-        <v>11.770491803278688</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="53">
+        <v>11.721311475409836</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="46">
         <v>15</v>
       </c>
       <c r="B18" s="28">
-        <v>1298</v>
+        <v>1290</v>
       </c>
       <c r="C18" s="29">
-        <v>1155</v>
+        <v>1153</v>
       </c>
       <c r="D18" s="27">
-        <v>88.983050847457619</v>
+        <v>89.379844961240309</v>
       </c>
       <c r="E18" s="27">
-        <v>-0.95550522013070349</v>
+        <v>0.39679411378268981</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G18" s="27">
-        <v>12.601941747572816</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="58" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19" s="58"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="58"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="58"/>
-    </row>
-    <row r="20" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="57" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="57"/>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
-      <c r="K20" s="51"/>
+        <v>12.524271844660195</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="62"/>
+      <c r="C19" s="62"/>
+      <c r="D19" s="62"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
+    </row>
+    <row r="20" spans="1:7" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="61"/>
+      <c r="C20" s="61"/>
+      <c r="D20" s="61"/>
+      <c r="E20" s="61"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="61"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2989,194 +2995,194 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:G20"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:K20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.88671875" customWidth="1"/>
-    <col min="2" max="4" width="11.33203125" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
-    <col min="6" max="6" width="12.5546875" customWidth="1"/>
-    <col min="7" max="7" width="12.109375" customWidth="1"/>
-    <col min="8" max="9" width="11.33203125" customWidth="1"/>
-    <col min="12" max="12" width="11.88671875" customWidth="1"/>
-    <col min="13" max="13" width="11.6640625" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="8" max="9" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.85546875" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="40.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="56" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="56"/>
-      <c r="C1" s="56"/>
-      <c r="D1" s="56"/>
-      <c r="E1" s="56"/>
-      <c r="F1" s="56"/>
-      <c r="G1" s="56"/>
-    </row>
-    <row r="2" spans="1:7" ht="51.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
-        <v>48</v>
-      </c>
-      <c r="B2" s="48" t="s">
+    <row r="1" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="60" t="s">
+        <v>54</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+    </row>
+    <row r="2" spans="1:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="49" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="48" t="s">
+      <c r="C2" s="49" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="48" t="s">
+      <c r="D2" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="49" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="F2" s="48" t="s">
-        <v>27</v>
-      </c>
-      <c r="G2" s="48" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="47" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" s="42">
-        <v>12936</v>
+        <v>12919</v>
       </c>
       <c r="C3" s="42">
-        <v>11843</v>
+        <v>11819</v>
       </c>
       <c r="D3" s="43">
-        <v>91.550711193568333</v>
-      </c>
-      <c r="E3" s="44" t="s">
-        <v>60</v>
+        <v>91.485409087390664</v>
+      </c>
+      <c r="E3" s="43">
+        <v>-6.5302106177668406E-2</v>
       </c>
       <c r="F3" s="44" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G3" s="44">
-        <v>13.850107066381156</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="45">
+        <v>13.831905781584583</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="54">
         <v>1</v>
       </c>
       <c r="B4" s="1">
-        <v>1896</v>
+        <v>1905</v>
       </c>
       <c r="C4" s="2">
-        <v>1657</v>
+        <v>1692</v>
       </c>
       <c r="D4" s="3">
-        <v>87.394514767932492</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>60</v>
+        <v>88.818897637795274</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1.4243828698627823</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G4" s="3">
-        <v>11.152941176470588</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="45">
+        <v>11.205882352941176</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="54">
         <v>2</v>
       </c>
       <c r="B5" s="1">
-        <v>750</v>
+        <v>747</v>
       </c>
       <c r="C5" s="2">
-        <v>710</v>
+        <v>696</v>
       </c>
       <c r="D5" s="3">
-        <v>94.666666666666671</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>60</v>
+        <v>93.172690763052216</v>
+      </c>
+      <c r="E5" s="3">
+        <v>-1.4939759036144551</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G5" s="3">
-        <v>12.096774193548388</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="45">
+        <v>12.048387096774194</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="54">
         <v>3</v>
       </c>
       <c r="B6" s="1">
-        <v>1249</v>
+        <v>1253</v>
       </c>
       <c r="C6" s="2">
-        <v>1173</v>
+        <v>1178</v>
       </c>
       <c r="D6" s="3">
-        <v>93.915132105684549</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>60</v>
+        <v>94.014365522745408</v>
+      </c>
+      <c r="E6" s="3">
+        <v>9.9233417060858642E-2</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G6" s="3">
-        <v>14.523255813953488</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="45">
+        <v>14.569767441860465</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="54">
         <v>4</v>
       </c>
       <c r="B7" s="1">
-        <v>722</v>
+        <v>718</v>
       </c>
       <c r="C7" s="2">
-        <v>641</v>
+        <v>640</v>
       </c>
       <c r="D7" s="3">
-        <v>88.78116343490305</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>60</v>
+        <v>89.136490250696383</v>
+      </c>
+      <c r="E7" s="3">
+        <v>0.35532681579333314</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G7" s="3">
-        <v>13.37037037037037</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" ht="11.25" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="45">
+        <v>13.296296296296296</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="54">
         <v>5</v>
       </c>
       <c r="B8" s="1">
-        <v>771</v>
+        <v>773</v>
       </c>
       <c r="C8" s="2">
-        <v>723</v>
+        <v>719</v>
       </c>
       <c r="D8" s="3">
-        <v>93.774319066147854</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>60</v>
+        <v>93.014230271668822</v>
+      </c>
+      <c r="E8" s="3">
+        <v>-0.76008879447903155</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G8" s="3">
-        <v>14.018181818181818</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="45">
+        <v>14.054545454545455</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="54">
         <v>6</v>
       </c>
       <c r="B9" s="1">
@@ -3188,64 +3194,64 @@
       <c r="D9" s="3">
         <v>96.174863387978135</v>
       </c>
-      <c r="E9" s="3" t="s">
-        <v>60</v>
+      <c r="E9" s="3">
+        <v>0</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G9" s="3">
         <v>12.620689655172415</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="45">
+    <row r="10" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="54">
         <v>7</v>
       </c>
       <c r="B10" s="1">
-        <v>1218</v>
+        <v>1203</v>
       </c>
       <c r="C10" s="2">
-        <v>1129</v>
+        <v>1124</v>
       </c>
       <c r="D10" s="3">
-        <v>92.692939244663393</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>60</v>
+        <v>93.433083956774738</v>
+      </c>
+      <c r="E10" s="3">
+        <v>0.74014471211134492</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G10" s="3">
-        <v>19.64516129032258</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="45">
+        <v>19.403225806451612</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="54">
         <v>8</v>
       </c>
       <c r="B11" s="1">
-        <v>511</v>
+        <v>512</v>
       </c>
       <c r="C11" s="2">
-        <v>454</v>
+        <v>446</v>
       </c>
       <c r="D11" s="3">
-        <v>88.845401174168288</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>60</v>
+        <v>87.109375</v>
+      </c>
+      <c r="E11" s="3">
+        <v>-1.7360261741682876</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G11" s="3">
-        <v>14.194444444444445</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="45">
+        <v>14.222222222222221</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="54">
         <v>9</v>
       </c>
       <c r="B12" s="1">
@@ -3257,175 +3263,179 @@
       <c r="D12" s="3">
         <v>89.179104477611943</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>60</v>
+      <c r="E12" s="3">
+        <v>0</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G12" s="3">
         <v>15.314285714285715</v>
       </c>
-    </row>
-    <row r="13" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="45">
+      <c r="I12" s="48"/>
+    </row>
+    <row r="13" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="54">
         <v>10</v>
       </c>
       <c r="B13" s="1">
-        <v>1162</v>
+        <v>1160</v>
       </c>
       <c r="C13" s="2">
-        <v>1084</v>
+        <v>1077</v>
       </c>
       <c r="D13" s="3">
-        <v>93.28743545611016</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>60</v>
+        <v>92.844827586206904</v>
+      </c>
+      <c r="E13" s="3">
+        <v>-0.44260786990325585</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G13" s="3">
-        <v>17.606060606060606</v>
-      </c>
-    </row>
-    <row r="14" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="45">
+        <v>17.575757575757574</v>
+      </c>
+      <c r="I13" s="48"/>
+    </row>
+    <row r="14" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="54">
         <v>11</v>
       </c>
       <c r="B14" s="1">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="C14" s="2">
-        <v>452</v>
+        <v>453</v>
       </c>
       <c r="D14" s="3">
-        <v>92.244897959183675</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>60</v>
+        <v>93.01848049281314</v>
+      </c>
+      <c r="E14" s="3">
+        <v>0.77358253362946527</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G14" s="3">
-        <v>15.806451612903226</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="45">
+        <v>15.709677419354838</v>
+      </c>
+      <c r="I14" s="48"/>
+    </row>
+    <row r="15" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="54">
         <v>12</v>
       </c>
       <c r="B15" s="1">
-        <v>398</v>
+        <v>397</v>
       </c>
       <c r="C15" s="2">
         <v>371</v>
       </c>
       <c r="D15" s="3">
-        <v>93.21608040201005</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>60</v>
+        <v>93.450881612090669</v>
+      </c>
+      <c r="E15" s="3">
+        <v>0.23480121008061872</v>
       </c>
       <c r="F15" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G15" s="3">
-        <v>15.92</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="45">
+        <v>15.88</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="54">
         <v>13</v>
       </c>
       <c r="B16" s="1">
-        <v>845</v>
+        <v>846</v>
       </c>
       <c r="C16" s="2">
-        <v>801</v>
+        <v>794</v>
       </c>
       <c r="D16" s="3">
-        <v>94.792899408284029</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>60</v>
+        <v>93.853427895981085</v>
+      </c>
+      <c r="E16" s="3">
+        <v>-0.93947151230294423</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G16" s="3">
-        <v>14.322033898305085</v>
-      </c>
-    </row>
-    <row r="17" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="45">
+        <v>14.338983050847459</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="54">
         <v>14</v>
       </c>
       <c r="B17" s="1">
-        <v>720</v>
+        <v>718</v>
       </c>
       <c r="C17" s="2">
-        <v>647</v>
+        <v>644</v>
       </c>
       <c r="D17" s="3">
-        <v>89.861111111111114</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>60</v>
+        <v>89.693593314763234</v>
+      </c>
+      <c r="E17" s="3">
+        <v>-0.16751779634788022</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G17" s="3">
-        <v>11.803278688524591</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="46">
+        <v>11.770491803278688</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="55">
         <v>15</v>
       </c>
       <c r="B18" s="28">
-        <v>1302</v>
+        <v>1298</v>
       </c>
       <c r="C18" s="29">
-        <v>1171</v>
+        <v>1155</v>
       </c>
       <c r="D18" s="27">
-        <v>89.938556067588323</v>
-      </c>
-      <c r="E18" s="27" t="s">
-        <v>60</v>
+        <v>88.983050847457619</v>
+      </c>
+      <c r="E18" s="27">
+        <v>-0.95550522013070349</v>
       </c>
       <c r="F18" s="27" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="G18" s="27">
-        <v>12.640776699029127</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A19" s="58" t="s">
-        <v>70</v>
-      </c>
-      <c r="B19" s="58"/>
-      <c r="C19" s="58"/>
-      <c r="D19" s="58"/>
-      <c r="E19" s="58"/>
-      <c r="F19" s="58"/>
-      <c r="G19" s="58"/>
-    </row>
-    <row r="20" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="57" t="s">
-        <v>36</v>
-      </c>
-      <c r="B20" s="57"/>
-      <c r="C20" s="57"/>
-      <c r="D20" s="57"/>
-      <c r="E20" s="57"/>
-      <c r="F20" s="57"/>
-      <c r="G20" s="57"/>
+        <v>12.601941747572816</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="62"/>
+      <c r="C19" s="62"/>
+      <c r="D19" s="62"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
+    </row>
+    <row r="20" spans="1:11" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="61"/>
+      <c r="C20" s="61"/>
+      <c r="D20" s="61"/>
+      <c r="E20" s="61"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="61"/>
+      <c r="K20" s="53"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -3439,31 +3449,484 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D39"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:I20"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="47.6640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="94.109375" style="36" customWidth="1"/>
-    <col min="3" max="3" width="92.88671875" customWidth="1"/>
+    <col min="1" max="1" width="13.85546875" customWidth="1"/>
+    <col min="2" max="4" width="11.28515625" customWidth="1"/>
+    <col min="5" max="5" width="15.7109375" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" customWidth="1"/>
+    <col min="7" max="7" width="12.140625" customWidth="1"/>
+    <col min="8" max="9" width="11.28515625" customWidth="1"/>
+    <col min="12" max="12" width="11.85546875" customWidth="1"/>
+    <col min="13" max="13" width="11.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="40.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="60" t="s">
+        <v>55</v>
+      </c>
+      <c r="B1" s="60"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="60"/>
+      <c r="E1" s="60"/>
+      <c r="F1" s="60"/>
+      <c r="G1" s="60"/>
+    </row>
+    <row r="2" spans="1:9" ht="51.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="49" t="s">
+        <v>46</v>
+      </c>
+      <c r="B2" s="49" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="49" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="49" t="s">
+        <v>44</v>
+      </c>
+      <c r="E2" s="49" t="s">
+        <v>43</v>
+      </c>
+      <c r="F2" s="49" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="49" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="47" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="42">
+        <v>12936</v>
+      </c>
+      <c r="C3" s="42">
+        <v>11843</v>
+      </c>
+      <c r="D3" s="43">
+        <v>91.550711193568333</v>
+      </c>
+      <c r="E3" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="F3" s="44" t="s">
+        <v>56</v>
+      </c>
+      <c r="G3" s="44">
+        <v>13.850107066381156</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="45">
+        <v>1</v>
+      </c>
+      <c r="B4" s="1">
+        <v>1896</v>
+      </c>
+      <c r="C4" s="2">
+        <v>1657</v>
+      </c>
+      <c r="D4" s="3">
+        <v>87.394514767932492</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="3">
+        <v>11.152941176470588</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="45">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1">
+        <v>750</v>
+      </c>
+      <c r="C5" s="2">
+        <v>710</v>
+      </c>
+      <c r="D5" s="3">
+        <v>94.666666666666671</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" s="3">
+        <v>12.096774193548388</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="45">
+        <v>3</v>
+      </c>
+      <c r="B6" s="1">
+        <v>1249</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1173</v>
+      </c>
+      <c r="D6" s="3">
+        <v>93.915132105684549</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F6" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G6" s="3">
+        <v>14.523255813953488</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="45">
+        <v>4</v>
+      </c>
+      <c r="B7" s="1">
+        <v>722</v>
+      </c>
+      <c r="C7" s="2">
+        <v>641</v>
+      </c>
+      <c r="D7" s="3">
+        <v>88.78116343490305</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F7" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" s="3">
+        <v>13.37037037037037</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="11.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="45">
+        <v>5</v>
+      </c>
+      <c r="B8" s="1">
+        <v>771</v>
+      </c>
+      <c r="C8" s="2">
+        <v>723</v>
+      </c>
+      <c r="D8" s="3">
+        <v>93.774319066147854</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F8" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G8" s="3">
+        <v>14.018181818181818</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="45">
+        <v>6</v>
+      </c>
+      <c r="B9" s="1">
+        <v>366</v>
+      </c>
+      <c r="C9" s="2">
+        <v>352</v>
+      </c>
+      <c r="D9" s="3">
+        <v>96.174863387978135</v>
+      </c>
+      <c r="E9" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F9" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" s="3">
+        <v>12.620689655172415</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A10" s="45">
+        <v>7</v>
+      </c>
+      <c r="B10" s="1">
+        <v>1218</v>
+      </c>
+      <c r="C10" s="2">
+        <v>1129</v>
+      </c>
+      <c r="D10" s="3">
+        <v>92.692939244663393</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F10" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G10" s="3">
+        <v>19.64516129032258</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="45">
+        <v>8</v>
+      </c>
+      <c r="B11" s="1">
+        <v>511</v>
+      </c>
+      <c r="C11" s="2">
+        <v>454</v>
+      </c>
+      <c r="D11" s="3">
+        <v>88.845401174168288</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F11" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="3">
+        <v>14.194444444444445</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A12" s="45">
+        <v>9</v>
+      </c>
+      <c r="B12" s="1">
+        <v>536</v>
+      </c>
+      <c r="C12" s="2">
+        <v>478</v>
+      </c>
+      <c r="D12" s="3">
+        <v>89.179104477611943</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F12" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G12" s="3">
+        <v>15.314285714285715</v>
+      </c>
+      <c r="I12" s="48"/>
+    </row>
+    <row r="13" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="45">
+        <v>10</v>
+      </c>
+      <c r="B13" s="1">
+        <v>1162</v>
+      </c>
+      <c r="C13" s="2">
+        <v>1084</v>
+      </c>
+      <c r="D13" s="3">
+        <v>93.28743545611016</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G13" s="3">
+        <v>17.606060606060606</v>
+      </c>
+      <c r="I13" s="48"/>
+    </row>
+    <row r="14" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="45">
+        <v>11</v>
+      </c>
+      <c r="B14" s="1">
+        <v>490</v>
+      </c>
+      <c r="C14" s="2">
+        <v>452</v>
+      </c>
+      <c r="D14" s="3">
+        <v>92.244897959183675</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="3">
+        <v>15.806451612903226</v>
+      </c>
+      <c r="I14" s="48"/>
+    </row>
+    <row r="15" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="45">
+        <v>12</v>
+      </c>
+      <c r="B15" s="1">
+        <v>398</v>
+      </c>
+      <c r="C15" s="2">
+        <v>371</v>
+      </c>
+      <c r="D15" s="3">
+        <v>93.21608040201005</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G15" s="3">
+        <v>15.92</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="45">
+        <v>13</v>
+      </c>
+      <c r="B16" s="1">
+        <v>845</v>
+      </c>
+      <c r="C16" s="2">
+        <v>801</v>
+      </c>
+      <c r="D16" s="3">
+        <v>94.792899408284029</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G16" s="3">
+        <v>14.322033898305085</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="45">
+        <v>14</v>
+      </c>
+      <c r="B17" s="1">
+        <v>720</v>
+      </c>
+      <c r="C17" s="2">
+        <v>647</v>
+      </c>
+      <c r="D17" s="3">
+        <v>89.861111111111114</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="G17" s="3">
+        <v>11.803278688524591</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="46">
+        <v>15</v>
+      </c>
+      <c r="B18" s="28">
+        <v>1302</v>
+      </c>
+      <c r="C18" s="29">
+        <v>1171</v>
+      </c>
+      <c r="D18" s="27">
+        <v>89.938556067588323</v>
+      </c>
+      <c r="E18" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="27" t="s">
+        <v>56</v>
+      </c>
+      <c r="G18" s="27">
+        <v>12.640776699029127</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="12" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="B19" s="62"/>
+      <c r="C19" s="62"/>
+      <c r="D19" s="62"/>
+      <c r="E19" s="62"/>
+      <c r="F19" s="62"/>
+      <c r="G19" s="62"/>
+    </row>
+    <row r="20" spans="1:7" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" s="61" t="s">
+        <v>35</v>
+      </c>
+      <c r="B20" s="61"/>
+      <c r="C20" s="61"/>
+      <c r="D20" s="61"/>
+      <c r="E20" s="61"/>
+      <c r="F20" s="61"/>
+      <c r="G20" s="61"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A19:G19"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="200" verticalDpi="200" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:G39"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="47.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="94.140625" style="36" customWidth="1"/>
+    <col min="3" max="3" width="92.85546875" customWidth="1"/>
     <col min="4" max="16384" width="11" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="59" t="s">
+    <row r="1" spans="1:4" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="63" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="60"/>
-    </row>
-    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="64"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
       <c r="B2" s="15" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>4</v>
       </c>
@@ -3471,7 +3934,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
@@ -3479,7 +3942,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>8</v>
       </c>
@@ -3487,39 +3950,39 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="8" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="52" t="s">
         <v>10</v>
       </c>
       <c r="B6" s="32" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:4" ht="42" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:4" ht="39" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="18" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B8" s="33" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="129.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="129.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
         <v>13</v>
       </c>
       <c r="B9" s="19" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
         <v>14</v>
       </c>
@@ -3527,7 +3990,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>16</v>
       </c>
@@ -3535,15 +3998,15 @@
         <v>9</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="52" t="s">
         <v>17</v>
       </c>
       <c r="B12" s="34" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="8" t="s">
         <v>11</v>
       </c>
@@ -3551,24 +4014,24 @@
         <v>33</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="35" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="27.6" x14ac:dyDescent="0.3">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="19" t="s">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D15" s="37"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="10" t="s">
         <v>14</v>
       </c>
@@ -3576,7 +4039,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="11" t="s">
         <v>16</v>
       </c>
@@ -3584,39 +4047,39 @@
         <v>9</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A18" s="8" t="s">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="52" t="s">
         <v>18</v>
       </c>
       <c r="B18" s="34" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B19" s="22" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
         <v>12</v>
       </c>
       <c r="B20" s="35" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
         <v>13</v>
       </c>
       <c r="B21" s="19" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="10" t="s">
         <v>14</v>
       </c>
@@ -3624,7 +4087,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" ht="20.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="11" t="s">
         <v>16</v>
       </c>
@@ -3632,39 +4095,39 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A24" s="8" t="s">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="52" t="s">
         <v>19</v>
       </c>
       <c r="B24" s="17" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="28.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A25" s="8" t="s">
         <v>11</v>
       </c>
       <c r="B25" s="25" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B26" s="49" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="27.6" x14ac:dyDescent="0.3">
+      <c r="B26" s="50" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A27" s="10" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="19" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="10" t="s">
         <v>14</v>
       </c>
@@ -3672,94 +4135,51 @@
         <v>15</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="11" t="s">
         <v>16</v>
       </c>
       <c r="B29" s="24" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A30" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B30" s="34" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="8" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31" s="22" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A32" s="9" t="s">
-        <v>12</v>
-      </c>
-      <c r="B32" s="35" t="s">
-        <v>68</v>
-      </c>
-      <c r="D32" s="31"/>
-    </row>
-    <row r="33" spans="1:2" ht="41.4" x14ac:dyDescent="0.3">
-      <c r="A33" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="B33" s="19" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A34" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B34" s="23" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="35" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A35" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="B35" s="24" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" s="26" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="36" spans="1:2" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B36" s="26" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="37" spans="1:2" ht="34.950000000000003" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="6" t="s">
+    <row r="31" spans="1:2" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B37" s="26" t="s">
+      <c r="B31" s="26" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A38" s="7" t="s">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="B38" s="17" t="s">
+      <c r="B32" s="17" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="39" spans="1:2" ht="49.95" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="12" t="s">
+    <row r="33" spans="1:7" ht="40.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A33" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B39" s="41" t="s">
-        <v>37</v>
-      </c>
+      <c r="B33" s="41" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="D39" s="31"/>
+      <c r="E39" s="31"/>
+      <c r="F39" s="31"/>
+      <c r="G39" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>